<commit_message>
Plotting against one individual
</commit_message>
<xml_diff>
--- a/Parameters/PFAS_parameters.xlsx
+++ b/Parameters/PFAS_parameters.xlsx
@@ -14194,19 +14194,18 @@
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="118234e2-ac85-44d7-a055-e5c370c0519f">
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="568ff3df-f16a-482d-bb3c-58af1efa1658">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="02553e5c-4019-4e05-9d39-79473b436dc7" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100094B3BF347DFD7448D6D53FC91363B33" ma:contentTypeVersion="16" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d1cd2a34398d9e4c261437f1aeee2bf3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="118234e2-ac85-44d7-a055-e5c370c0519f" xmlns:ns3="02553e5c-4019-4e05-9d39-79473b436dc7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="625a357b965783487785174984a1a796" ns2:_="" ns3:_="">
-    <xsd:import namespace="118234e2-ac85-44d7-a055-e5c370c0519f"/>
-    <xsd:import namespace="02553e5c-4019-4e05-9d39-79473b436dc7"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002AA8BEAC825CAE4DA772B4C276EF423C" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="5e03e074850d6c738b9d1fc41fb3a339">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="568ff3df-f16a-482d-bb3c-58af1efa1658" xmlns:ns3="13cea704-446d-46be-be94-9e10425fef80" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="54949abb9ca0b8b43f171cb19b04d06d" ns2:_="" ns3:_="">
+    <xsd:import namespace="568ff3df-f16a-482d-bb3c-58af1efa1658"/>
+    <xsd:import namespace="13cea704-446d-46be-be94-9e10425fef80"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -14215,16 +14214,13 @@
               <xsd:all>
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
                 <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
               </xsd:all>
@@ -14234,7 +14230,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="118234e2-ac85-44d7-a055-e5c370c0519f" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="568ff3df-f16a-482d-bb3c-58af1efa1658" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -14247,60 +14243,50 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="c7855947-2042-4236-af9d-b08e54de1c70" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="11" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="5ec99919-4982-4388-8a64-83a11d2ca210" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="20" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="12" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="21" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="13" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+    <xsd:element name="MediaServiceEventHashCode" ma:index="14" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="17" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="18" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="19" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="02553e5c-4019-4e05-9d39-79473b436dc7" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="13cea704-446d-46be-be94-9e10425fef80" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Partagé avec" ma:hidden="true" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="15" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -14319,21 +14305,12 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Partagé avec détails" ma:hidden="true" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="16" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
       </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{7932d046-aa1e-4b99-8c82-0c2b73fc917d}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="02553e5c-4019-4e05-9d39-79473b436dc7">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -14345,8 +14322,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:displayName="Type de contenu"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="0" ma:displayName="Titre"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -14462,22 +14439,7 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD7061AE-6412-44F7-A40B-EAE36C498C4C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="118234e2-ac85-44d7-a055-e5c370c0519f"/>
-    <ds:schemaRef ds:uri="02553e5c-4019-4e05-9d39-79473b436dc7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0835BDDE-DE7E-41E6-9129-523C6A230D8C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>